<commit_message>
first new tree gauge implementation
</commit_message>
<xml_diff>
--- a/tests/coil_3D_avoltemf_edge/input_template.xlsx
+++ b/tests/coil_3D_avoltemf_edge/input_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
@@ -177,7 +177,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,12 +188,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -225,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -240,22 +234,13 @@
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -563,7 +548,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="14.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="14.862142857142858" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -575,7 +560,7 @@
       <c r="A1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>44</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -665,7 +650,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="3"/>
-      <c r="B5" s="9"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -727,15 +712,15 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -971,13 +956,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="3">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="D2" s="3">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E2" s="3">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F2" s="3">
         <v>0</v>
@@ -986,16 +971,16 @@
         <v>0</v>
       </c>
       <c r="H2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="3">
         <v>0</v>
       </c>
       <c r="J2" s="3">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
updates for edge elements new tree gauge algorithm
</commit_message>
<xml_diff>
--- a/tests/coil_3D_avoltemf_edge/input_template.xlsx
+++ b/tests/coil_3D_avoltemf_edge/input_template.xlsx
@@ -778,13 +778,13 @@
         <v>1</v>
       </c>
       <c r="H2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -810,13 +810,13 @@
         <v>3e-7</v>
       </c>
       <c r="H3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
@@ -842,13 +842,13 @@
         <v>2e-8</v>
       </c>
       <c r="H4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -962,7 +962,7 @@
         <v>2000</v>
       </c>
       <c r="E2" s="3">
-        <v>12</v>
+        <v>0.12566370614359</v>
       </c>
       <c r="F2" s="3">
         <v>0</v>
@@ -980,7 +980,7 @@
         <v>20</v>
       </c>
       <c r="K2" s="3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L2" s="3">
         <v>0</v>

</xml_diff>